<commit_message>
duplicate table issue fix
</commit_message>
<xml_diff>
--- a/low_risk_orange_results.xlsx
+++ b/low_risk_orange_results.xlsx
@@ -866,23 +866,23 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>066001876</t>
+          <t>420714325</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>2024</v>
       </c>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>City of New Haven</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>No FAC report found for EIN 066001876 in 2024.</t>
-        </is>
-      </c>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">

</xml_diff>